<commit_message>
Hesap DXF: her hesap ayrı çerçevede, yağmur notu kaldırıldı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/hesaplar_sema/HESAPLAR_SIHHI.xlsx
+++ b/proje/hesaplar_sema/HESAPLAR_SIHHI.xlsx
@@ -9748,7 +9748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -9945,13 +9945,6 @@
         <v/>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>*Yağmur suyu pis su kanalına bağlanmayacak, yağmur suyu kanalına (rögarına) verilecektir.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>